<commit_message>
refactor: core/cost_model.py fonte unica — PPTX e Excel consistentes
</commit_message>
<xml_diff>
--- a/docs/Custos_OmniChannel_Executivo.xlsx
+++ b/docs/Custos_OmniChannel_Executivo.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalhe" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projeções" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Mercado BR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projecoes Detalhe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Mercado BR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infra + IA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +25,7 @@
     <numFmt numFmtId="166" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,11 +64,6 @@
     <font>
       <b val="1"/>
       <color rgb="00333333"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="004472C4"/>
       <sz val="11"/>
     </font>
     <font>
@@ -113,10 +108,6 @@
       <b val="1"/>
       <color rgb="00006100"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
     </font>
   </fonts>
   <fills count="5">
@@ -163,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,6 +174,9 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -195,22 +189,16 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -219,17 +207,14 @@
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -237,13 +222,13 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -252,81 +237,77 @@
     <xf numFmtId="3" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -693,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -702,26 +683,27 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOS OMNI CHANNEL · Infra + IA (Desenvolvimento + Produção)</t>
+          <t>CUSTOS OMNI CHANNEL · Infra + IA (Dev + Producao)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>13/07/2026 03:07 | R$5.50/USD | Margem 10% | DeepSeek pay-per-token | MiniMax Plus $20/mês | Valores em BRL</t>
+          <t>13/07/2026 03:48 | R$5.50/USD | 10% margem | DeepSeek pay-per-token | MiniMax Plus $20/mes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>HOJE — Custo Operacional Real</t>
+          <t>HOJE — Custo Operacional (recorrente 24/7)</t>
         </is>
       </c>
     </row>
@@ -733,17 +715,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Serviço</t>
+          <t>Servico</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>USD/mês</t>
+          <t>USD/mes</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BRL/mês</t>
+          <t>BRL/mes</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -753,7 +735,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Descrição</t>
+          <t>Tipo</t>
         </is>
       </c>
     </row>
@@ -765,7 +747,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Worker (4vCPU/4GB, min=1)</t>
+          <t>Cloud Run Worker (4vCPU/4GB, min=1, 730h/mes)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -777,9 +759,9 @@
       <c r="E6" s="8" t="n">
         <v>0.4060681232706803</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -791,7 +773,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>API + Portal Cloud Run (min=0)</t>
+          <t>API + Portal Cloud Run (min=0, idle)</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -803,9 +785,9 @@
       <c r="E7" s="8" t="n">
         <v>0.03673313615113061</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -817,7 +799,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Firestore (2 projetos)</t>
+          <t>Firestore (2 projetos: chamadas + WhatsApp)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -829,9 +811,9 @@
       <c r="E8" s="8" t="n">
         <v>0.07871386318099417</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -843,7 +825,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Cloud Storage (audios + backups)</t>
+          <t>Cloud Storage (audios temporarios + backups)</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -855,9 +837,9 @@
       <c r="E9" s="8" t="n">
         <v>0.03148554527239767</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -869,7 +851,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pub/Sub + Secret Manager</t>
+          <t>Pub/Sub + Secret Manager (10 secrets)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -881,9 +863,9 @@
       <c r="E10" s="8" t="n">
         <v>0.01574277263619884</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -895,7 +877,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Cloud Build + Artifact Registry</t>
+          <t>Cloud Build + Artifact Registry (CI/CD)</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -907,9 +889,9 @@
       <c r="E11" s="8" t="n">
         <v>0.02099036351493178</v>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
@@ -921,7 +903,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>VM e2-small + IP (WhatsApp)</t>
+          <t>VM e2-small + IP WhatsApp (Evolution API)</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -933,21 +915,21 @@
       <c r="E12" s="8" t="n">
         <v>0.1049518175746589</v>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Infraestrutura cloud</t>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Infra</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>IA Desenv.</t>
+          <t>IA Dev</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>DeepSeek — tokens desenvolvimento (testes, prompts)</t>
+          <t>DeepSeek V4 Flash — Desenvolvimento (testes, prompts, engenharia)</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -959,21 +941,21 @@
       <c r="E13" s="8" t="n">
         <v>0.07871386318099417</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>LLM API</t>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>IA Desenv.</t>
+          <t>IA Dev</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>MiniMax Plus — plano mensal (fallback + créditos)</t>
+          <t>MiniMax Plus — Plano fixo mensal ($20/mes, fallback + creditos)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -985,21 +967,21 @@
       <c r="E14" s="8" t="n">
         <v>0.09541074324968991</v>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>LLM API</t>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>IA Produção</t>
+          <t>IA Prod</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>DeepSeek — Monitoria (~20 chamadas/dia)</t>
+          <t>DeepSeek V4 Flash — Monitoria de Chamadas (~20 chamadas/dia)</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -1011,21 +993,21 @@
       <c r="E15" s="8" t="n">
         <v>0.01049518175746589</v>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>LLM API</t>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>IA Produção</t>
+          <t>IA Prod</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>DeepSeek — Chatbots WhatsApp (5 bots)</t>
+          <t>DeepSeek V4 Flash — Chatbots WhatsApp (5 bots, 200 msg/dia)</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -1037,21 +1019,21 @@
       <c r="E16" s="8" t="n">
         <v>0.04198072702986357</v>
       </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>LLM API</t>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>IA Produção</t>
+          <t>IA Prod</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>DeepSeek — Extras (URA dev, overflow)</t>
+          <t>DeepSeek V4 Flash — Extras (URA dev, overflow, melhorias)</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
@@ -1063,62 +1045,59 @@
       <c r="E17" s="8" t="n">
         <v>0.07871386318099417</v>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>LLM API</t>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>LLM</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>GCP Infraestrutura</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="n">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>GCP Infra</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
         <v>145.62</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="12" t="n">
         <v>800.9100000000001</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="13" t="n">
         <v>0.6946856216009922</v>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>IA Desenvolvimento</t>
         </is>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <v>36.5</v>
       </c>
-      <c r="D19" s="11" t="n">
+      <c r="D19" s="12" t="n">
         <v>200.75</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="13" t="n">
         <v>0.1741246064306841</v>
       </c>
-      <c r="F19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>IA Produção</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="n">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>IA Producao</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
         <v>27.5</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D20" s="12" t="n">
         <v>151.25</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="13" t="n">
         <v>0.1311897719683236</v>
       </c>
-      <c r="F20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -1137,29 +1116,28 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>PROJEÇÕES DE CRESCIMENTO — IA escala com volume de chamadas</t>
+          <t>PROJECOES DE CRESCIMENTO — Custo por volume de chamadas</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Cenário</t>
+          <t>Cenario</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Chamadas/mês</t>
+          <t>Chamadas/mes</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>GCP+IA/mês (BRL)</t>
+          <t>Total/mes (BRL)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1169,91 +1147,93 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Crescimento vs Hoje</t>
+          <t>GCP</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>IA Dev</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>IA Prod</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>500/dia (15,000/mês)</t>
-        </is>
-      </c>
-      <c r="B25" s="20" t="n">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>500/dia (15,000/mes)</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n">
         <v>15000</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C25" s="20" t="n">
         <v>1143.725</v>
       </c>
-      <c r="D25" s="22" t="n">
+      <c r="D25" s="21" t="n">
         <v>0.07624833333333332</v>
       </c>
-      <c r="E25" s="23" t="inlineStr">
-        <is>
-          <t>-1%</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>IA escala com volume, GCP infra otimizada</t>
-        </is>
+      <c r="E25" s="22" t="n">
+        <v>734.415</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>200.75</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>208.56</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="25" t="inlineStr">
-        <is>
-          <t>1000/dia (30,000/mês)</t>
-        </is>
-      </c>
-      <c r="B26" s="26" t="n">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>1000/dia (30,000/mes)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="n">
         <v>30000</v>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C26" s="25" t="n">
         <v>1252.46</v>
       </c>
-      <c r="D26" s="28" t="n">
+      <c r="D26" s="26" t="n">
         <v>0.04174866666666667</v>
       </c>
-      <c r="E26" s="29" t="inlineStr">
-        <is>
-          <t>+9%</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>IA escala com volume, GCP infra otimizada</t>
-        </is>
+      <c r="E26" s="27" t="n">
+        <v>778.5250000000001</v>
+      </c>
+      <c r="F26" s="27" t="n">
+        <v>200.75</v>
+      </c>
+      <c r="G26" s="27" t="n">
+        <v>273.185</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>5000/dia (150,000/mês)</t>
-        </is>
-      </c>
-      <c r="B27" s="31" t="n">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>5000/dia (150,000/mes)</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n">
         <v>150000</v>
       </c>
-      <c r="C27" s="32" t="n">
+      <c r="C27" s="30" t="n">
         <v>2121.955</v>
       </c>
-      <c r="D27" s="33" t="n">
+      <c r="D27" s="31" t="n">
         <v>0.01414636666666667</v>
       </c>
-      <c r="E27" s="34" t="inlineStr">
-        <is>
-          <t>+84%</t>
-        </is>
-      </c>
-      <c r="F27" s="35" t="inlineStr">
-        <is>
-          <t>IA escala com volume, GCP infra otimizada</t>
-        </is>
+      <c r="E27" s="32" t="n">
+        <v>1131.35</v>
+      </c>
+      <c r="F27" s="32" t="n">
+        <v>200.75</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <v>789.8549999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1268,398 +1248,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="004472C4"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>DETALHE COMPLETO — GCP Infra + IA (Dev + Produção)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>MiniMax Plus: plano fixo de $20/mês. DeepSeek: pay-per-token, sem plano fixo. Margem 10% em todos valores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="37" t="inlineStr">
-        <is>
-          <t>INFRAESTRUTURA GCP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="38" t="inlineStr">
-        <is>
-          <t>Worker (4vCPU/4GB, min=1)</t>
-        </is>
-      </c>
-      <c r="B5" s="39" t="n">
-        <v>77.38</v>
-      </c>
-      <c r="C5" s="39" t="n">
-        <v>85.12</v>
-      </c>
-      <c r="D5" s="40" t="n">
-        <v>468.16</v>
-      </c>
-      <c r="E5" s="41" t="inlineStr">
-        <is>
-          <t>IA Token</t>
-        </is>
-      </c>
-      <c r="F5" s="42" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
-        <is>
-          <t>API + Portal Cloud Run (min=0)</t>
-        </is>
-      </c>
-      <c r="B6" s="44" t="n">
-        <v>7</v>
-      </c>
-      <c r="C6" s="44" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="D6" s="45" t="n">
-        <v>42.35</v>
-      </c>
-      <c r="E6" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
-        <is>
-          <t>Firestore (2 projetos)</t>
-        </is>
-      </c>
-      <c r="B7" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="C7" s="44" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="D7" s="45" t="n">
-        <v>90.75</v>
-      </c>
-      <c r="E7" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>Cloud Storage (audios + backups)</t>
-        </is>
-      </c>
-      <c r="B8" s="44" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="44" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="D8" s="45" t="n">
-        <v>36.3</v>
-      </c>
-      <c r="E8" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="43" t="inlineStr">
-        <is>
-          <t>Pub/Sub + Secret Manager</t>
-        </is>
-      </c>
-      <c r="B9" s="44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="44" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="D9" s="45" t="n">
-        <v>18.15</v>
-      </c>
-      <c r="E9" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="43" t="inlineStr">
-        <is>
-          <t>Cloud Build + Artifact Registry</t>
-        </is>
-      </c>
-      <c r="B10" s="44" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="44" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="D10" s="45" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E10" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
-        <is>
-          <t>VM e2-small + IP (WhatsApp)</t>
-        </is>
-      </c>
-      <c r="B11" s="44" t="n">
-        <v>20</v>
-      </c>
-      <c r="C11" s="44" t="n">
-        <v>22</v>
-      </c>
-      <c r="D11" s="45" t="n">
-        <v>121</v>
-      </c>
-      <c r="E11" s="46" t="inlineStr">
-        <is>
-          <t>GCP</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="47" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B12" s="48" t="inlineStr"/>
-      <c r="C12" s="49" t="n">
-        <v>145.62</v>
-      </c>
-      <c r="D12" s="50" t="n">
-        <v>800.9100000000001</v>
-      </c>
-      <c r="E12" s="48" t="inlineStr"/>
-      <c r="F12" s="48" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="37" t="inlineStr">
-        <is>
-          <t>IA — DESENVOLVIMENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="38" t="inlineStr">
-        <is>
-          <t>DeepSeek — tokens desenvolvimento (testes, prompts)</t>
-        </is>
-      </c>
-      <c r="B15" s="39" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" s="39" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="D15" s="40" t="n">
-        <v>90.75</v>
-      </c>
-      <c r="E15" s="41" t="inlineStr">
-        <is>
-          <t>IA Token</t>
-        </is>
-      </c>
-      <c r="F15" s="42" t="inlineStr"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>MiniMax Plus — plano mensal (fallback + créditos)</t>
-        </is>
-      </c>
-      <c r="B16" s="44" t="n">
-        <v>20</v>
-      </c>
-      <c r="C16" s="44" t="n">
-        <v>20</v>
-      </c>
-      <c r="D16" s="45" t="n">
-        <v>110</v>
-      </c>
-      <c r="E16" s="46" t="inlineStr">
-        <is>
-          <t>Plano</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="47" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B17" s="48" t="inlineStr"/>
-      <c r="C17" s="49" t="n">
-        <v>36.5</v>
-      </c>
-      <c r="D17" s="50" t="n">
-        <v>200.75</v>
-      </c>
-      <c r="E17" s="48" t="inlineStr"/>
-      <c r="F17" s="48" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="37" t="inlineStr">
-        <is>
-          <t>IA — PRODUÇÃO (Módulos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="38" t="inlineStr">
-        <is>
-          <t>DeepSeek — Monitoria (~20 chamadas/dia)</t>
-        </is>
-      </c>
-      <c r="B20" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" s="39" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="D20" s="40" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="E20" s="41" t="inlineStr">
-        <is>
-          <t>IA Token</t>
-        </is>
-      </c>
-      <c r="F20" s="42" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="43" t="inlineStr">
-        <is>
-          <t>DeepSeek — Chatbots WhatsApp (5 bots)</t>
-        </is>
-      </c>
-      <c r="B21" s="44" t="n">
-        <v>8</v>
-      </c>
-      <c r="C21" s="44" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="D21" s="45" t="n">
-        <v>48.40000000000001</v>
-      </c>
-      <c r="E21" s="46" t="inlineStr">
-        <is>
-          <t>IA Token</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="43" t="inlineStr">
-        <is>
-          <t>DeepSeek — Extras (URA dev, overflow)</t>
-        </is>
-      </c>
-      <c r="B22" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" s="44" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="D22" s="45" t="n">
-        <v>90.75</v>
-      </c>
-      <c r="E22" s="46" t="inlineStr">
-        <is>
-          <t>IA Token</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="47" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B23" s="48" t="inlineStr"/>
-      <c r="C23" s="49" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="D23" s="50" t="n">
-        <v>151.25</v>
-      </c>
-      <c r="E23" s="48" t="inlineStr"/>
-      <c r="F23" s="48" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="51" t="inlineStr">
-        <is>
-          <t>TOTAL MENSAL</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="n">
-        <v>209.62</v>
-      </c>
-      <c r="D25" s="52" t="n">
-        <v>1152.91</v>
-      </c>
-      <c r="E25" s="18" t="inlineStr"/>
-      <c r="F25" s="18" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -1677,16 +1265,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>PROJEÇÕES DE CRESCIMENTO — DeepSeek primário + MiniMax Plus fallback</t>
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>PROJECOES DETALHADAS — Todos os componentes por cenario</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IA Desenvolvimento estabiliza. IA Produção escala com volume de chamadas. WhatsApp 5 bots incluso.</t>
+          <t>Valores em BRL com 10% de margem. WhatsApp 5 bots incluso nos 3 cenarios.</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1306,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="53" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>GCP — Worker (PUSH, min=0)</t>
         </is>
@@ -1732,14 +1320,14 @@
       <c r="D5" s="7" t="n">
         <v>441.045</v>
       </c>
-      <c r="E5" s="46" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="53" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>GCP — API+Storage+PubSub</t>
         </is>
@@ -1753,16 +1341,16 @@
       <c r="D6" s="7" t="n">
         <v>139.755</v>
       </c>
-      <c r="E6" s="46" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="53" t="inlineStr">
-        <is>
-          <t>GCP — WhatsApp 5 bots (Cloud Run+SQL)</t>
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>GCP — WhatsApp 5 bots</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -1774,16 +1362,16 @@
       <c r="D7" s="7" t="n">
         <v>550.55</v>
       </c>
-      <c r="E7" s="46" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Infra</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>IA Dev — DeepSeek (testes, prompts)</t>
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>IA Dev — DeepSeek (testes)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
@@ -1795,14 +1383,14 @@
       <c r="D8" s="7" t="n">
         <v>90.75</v>
       </c>
-      <c r="E8" s="46" t="inlineStr">
-        <is>
-          <t>IA Desenv.</t>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>IA Dev</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="53" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>IA Dev — MiniMax Plus plano</t>
         </is>
@@ -1816,16 +1404,16 @@
       <c r="D9" s="7" t="n">
         <v>110</v>
       </c>
-      <c r="E9" s="46" t="inlineStr">
-        <is>
-          <t>IA Desenv.</t>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>IA Dev</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="53" t="inlineStr">
-        <is>
-          <t>IA Prod — DeepSeek Monitoria (diariz+QA)</t>
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>IA Prod — DeepSeek Monitoria</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -1837,14 +1425,14 @@
       <c r="D10" s="7" t="n">
         <v>622.545</v>
       </c>
-      <c r="E10" s="46" t="inlineStr">
-        <is>
-          <t>IA Produção</t>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>IA Prod</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="53" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
         <is>
           <t>IA Prod — DeepSeek Chatbots</t>
         </is>
@@ -1858,16 +1446,16 @@
       <c r="D11" s="7" t="n">
         <v>53.23999999999999</v>
       </c>
-      <c r="E11" s="46" t="inlineStr">
-        <is>
-          <t>IA Produção</t>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>IA Prod</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="53" t="inlineStr">
-        <is>
-          <t>IA Prod — DeepSeek Extras (URA dev)</t>
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>IA Prod — DeepSeek Extras</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -1879,16 +1467,16 @@
       <c r="D12" s="7" t="n">
         <v>90.75</v>
       </c>
-      <c r="E12" s="46" t="inlineStr">
-        <is>
-          <t>IA Produção</t>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>IA Prod</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="53" t="inlineStr">
-        <is>
-          <t>IA Prod — MiniMax fallback (5%)</t>
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>IA Prod — MiniMax fallback</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -1900,93 +1488,93 @@
       <c r="D13" s="7" t="n">
         <v>23.32</v>
       </c>
-      <c r="E13" s="46" t="inlineStr">
-        <is>
-          <t>IA Produção</t>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>IA Prod</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="47" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>TOTAL GCP</t>
         </is>
       </c>
-      <c r="B14" s="50" t="n">
+      <c r="B14" s="36" t="n">
         <v>734.415</v>
       </c>
-      <c r="C14" s="50" t="n">
+      <c r="C14" s="36" t="n">
         <v>778.5250000000001</v>
       </c>
-      <c r="D14" s="50" t="n">
+      <c r="D14" s="36" t="n">
         <v>1131.35</v>
       </c>
-      <c r="E14" s="48" t="inlineStr"/>
+      <c r="E14" s="37" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="47" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>TOTAL IA Desenvolvimento</t>
         </is>
       </c>
-      <c r="B15" s="50" t="n">
+      <c r="B15" s="36" t="n">
         <v>200.75</v>
       </c>
-      <c r="C15" s="50" t="n">
+      <c r="C15" s="36" t="n">
         <v>200.75</v>
       </c>
-      <c r="D15" s="50" t="n">
+      <c r="D15" s="36" t="n">
         <v>200.75</v>
       </c>
-      <c r="E15" s="48" t="inlineStr"/>
+      <c r="E15" s="37" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="47" t="inlineStr">
-        <is>
-          <t>TOTAL IA Produção</t>
-        </is>
-      </c>
-      <c r="B16" s="50" t="n">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>TOTAL IA Producao</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n">
         <v>208.56</v>
       </c>
-      <c r="C16" s="50" t="n">
+      <c r="C16" s="36" t="n">
         <v>273.185</v>
       </c>
-      <c r="D16" s="50" t="n">
+      <c r="D16" s="36" t="n">
         <v>789.8549999999999</v>
       </c>
-      <c r="E16" s="48" t="inlineStr"/>
+      <c r="E16" s="37" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="51" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL MENSAL</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="n">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>CUSTO TOTAL</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
         <v>1143.725</v>
       </c>
-      <c r="C17" s="32" t="n">
+      <c r="C17" s="30" t="n">
         <v>1252.46</v>
       </c>
-      <c r="D17" s="32" t="n">
+      <c r="D17" s="30" t="n">
         <v>2121.955</v>
       </c>
-      <c r="E17" s="18" t="inlineStr"/>
+      <c r="E17" s="39" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="54" t="inlineStr">
+      <c r="A19" s="40" t="inlineStr">
         <is>
           <t>Custo por Chamada</t>
         </is>
       </c>
-      <c r="B19" s="28" t="n">
+      <c r="B19" s="26" t="n">
         <v>0.07624833333333332</v>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="26" t="n">
         <v>0.04174866666666667</v>
       </c>
-      <c r="D19" s="28" t="n">
+      <c r="D19" s="26" t="n">
         <v>0.01414636666666667</v>
       </c>
     </row>
@@ -1999,36 +1587,35 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>COMPARATIVO — Operações Nacionais (Brasil)</t>
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>COMPARATIVO — Operadoras Nacionais (Brasil)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nossa solução (500 chamadas/dia): R$ 0.08/chamada, automatizada. Operadoras tradicionais: QA humano, R$ 0,30-1,00/chamada.</t>
+          <t>Nossa solucao: R$ 0.08/chamada (500/dia). Trade: QA humano — amostragem 2-5% vs 100% automatizado.</t>
         </is>
       </c>
     </row>
@@ -2050,12 +1637,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Custo QA/chamada</t>
+          <t>Custo/chamada</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>vs Nós</t>
+          <t>vs Nos</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2063,212 +1650,499 @@
           <t>Nossa Vantagem</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="25" t="inlineStr">
-        <is>
-          <t>Teleperformance (Brasil)</t>
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Teleperformance Brasil</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>BPO global, 80K funcionários BR</t>
+          <t>BPO global, 80 mil funcionarios no Brasil</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>QA humano por amostragem</t>
-        </is>
-      </c>
-      <c r="D5" s="55" t="inlineStr">
+          <t>QA humano — analistas escutam amostras (2-5% das chamadas)</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>R$ 0.50–1.00</t>
         </is>
       </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>10x mais caro</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Automatizavel — R$ 0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Atento Brasil</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Maior BPO da America Latina, 90 mil func. BR</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Monitoria manual — equipe dedicada de qualidade</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>R$ 0.40–0.80</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>8x mais caro</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Automatizavel — R$ 0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>NOSSA (500/dia)</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>OmniChannel</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>IA — 100% automatizado</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>R$ 0.08</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>NOSSA (5.000/dia)</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>OmniChannel</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>IA — 100% automatizado</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>R$ 0.01</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>DETALHE COMPLETO — Todos os servicos GCP + LLM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="46" t="inlineStr">
+        <is>
+          <t>INFRAESTRUTURA GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Cloud Run Worker (4vCPU/4GB, min=1, 730h/mes)</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="n">
+        <v>77.38</v>
+      </c>
+      <c r="C4" s="48" t="n">
+        <v>85.12</v>
+      </c>
+      <c r="D4" s="49" t="n">
+        <v>468.16</v>
+      </c>
+      <c r="E4" s="50" t="inlineStr">
+        <is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="51" t="inlineStr">
+        <is>
+          <t>API + Portal Cloud Run (min=0, idle)</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" s="52" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>42.35</v>
+      </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>10x mais caro</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Automatizável — nosso custo R$ 0.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>Atento (Brasil)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Maior BPO LatAm, 90K func. BR</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Monitoria manual de chamadas</t>
-        </is>
-      </c>
-      <c r="D6" s="55" t="inlineStr">
-        <is>
-          <t>R$ 0.40–0.80</t>
-        </is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="51" t="inlineStr">
+        <is>
+          <t>Firestore (2 projetos: chamadas + WhatsApp)</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="52" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>90.75</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>8x mais caro</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Automatizável — nosso custo R$ 0.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t>Liq (Bertelsmann)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>BPO digital, 40K func. BR</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Plataforma própria + terceiros</t>
-        </is>
-      </c>
-      <c r="D7" s="55" t="inlineStr">
-        <is>
-          <t>R$ 0.35–0.70</t>
-        </is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="51" t="inlineStr">
+        <is>
+          <t>Cloud Storage (audios temporarios + backups)</t>
+        </is>
+      </c>
+      <c r="B7" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="52" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>36.3</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>7x mais caro</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Automatizável — nosso custo R$ 0.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>Algar Tech</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>BPO médio, 20K func. BR</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Soluções híbridas</t>
-        </is>
-      </c>
-      <c r="D8" s="55" t="inlineStr">
-        <is>
-          <t>R$ 0.30–0.60</t>
-        </is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="51" t="inlineStr">
+        <is>
+          <t>Pub/Sub + Secret Manager (10 secrets)</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="52" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <v>18.15</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>6x mais caro</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Automatizável — nosso custo R$ 0.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="56" t="inlineStr">
-        <is>
-          <t>NOSSA SOLUÇÃO (500/dia)</t>
-        </is>
-      </c>
-      <c r="B9" s="35" t="inlineStr">
-        <is>
-          <t>OmniChannel</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>IA — sem intervenção humana</t>
-        </is>
-      </c>
-      <c r="D9" s="57" t="inlineStr">
-        <is>
-          <t>R$ 0.08</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>Referência</t>
-        </is>
-      </c>
-      <c r="F9" s="35" t="inlineStr">
-        <is>
-          <t>QA 100% automatizado — DeepSeek V4 Flash</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="56" t="inlineStr">
-        <is>
-          <t>NOSSA SOLUÇÃO (5.000/dia)</t>
-        </is>
-      </c>
-      <c r="B10" s="35" t="inlineStr">
-        <is>
-          <t>OmniChannel</t>
-        </is>
-      </c>
-      <c r="C10" s="35" t="inlineStr">
-        <is>
-          <t>IA — sem intervenção humana</t>
-        </is>
-      </c>
-      <c r="D10" s="57" t="inlineStr">
-        <is>
-          <t>R$ 0.01</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>Referência</t>
-        </is>
-      </c>
-      <c r="F10" s="35" t="inlineStr">
-        <is>
-          <t>Escala reduz custo por chamada</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="58" t="inlineStr">
-        <is>
-          <t>Nosso custo de QA automatizado é 5-17x menor que o custo de QA humano das operadoras nacionais.</t>
-        </is>
-      </c>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>Cloud Build + Artifact Registry (CI/CD)</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="52" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>VM e2-small + IP WhatsApp (Evolution API)</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="52" t="n">
+        <v>22</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="inlineStr"/>
+      <c r="C11" s="53" t="n">
+        <v>145.62</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>800.9100000000001</v>
+      </c>
+      <c r="E11" s="37" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>IA — DESENVOLVIMENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="47" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash — Desenvolvimento (testes, prompts, engenharia)</t>
+        </is>
+      </c>
+      <c r="B14" s="48" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="48" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D14" s="49" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="E14" s="50" t="inlineStr">
+        <is>
+          <t>IA Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="51" t="inlineStr">
+        <is>
+          <t>MiniMax Plus — Plano fixo mensal ($20/mes, fallback + creditos)</t>
+        </is>
+      </c>
+      <c r="B15" s="52" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" s="52" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>110</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Plano</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr"/>
+      <c r="C16" s="53" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>200.75</v>
+      </c>
+      <c r="E16" s="37" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="46" t="inlineStr">
+        <is>
+          <t>IA — PRODUCAO (Modulos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash — Monitoria de Chamadas (~20 chamadas/dia)</t>
+        </is>
+      </c>
+      <c r="B19" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="48" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D19" s="49" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="E19" s="50" t="inlineStr">
+        <is>
+          <t>IA Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="51" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash — Chatbots WhatsApp (5 bots, 200 msg/dia)</t>
+        </is>
+      </c>
+      <c r="B20" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" s="52" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <v>48.40000000000001</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>IA Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="51" t="inlineStr">
+        <is>
+          <t>DeepSeek V4 Flash — Extras (URA dev, overflow, melhorias)</t>
+        </is>
+      </c>
+      <c r="B21" s="52" t="n">
+        <v>15</v>
+      </c>
+      <c r="C21" s="52" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>IA Token</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B22" s="37" t="inlineStr"/>
+      <c r="C22" s="53" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D22" s="36" t="n">
+        <v>151.25</v>
+      </c>
+      <c r="E22" s="37" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL MENSAL</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>209.62</v>
+      </c>
+      <c r="D24" s="54" t="n">
+        <v>1152.91</v>
+      </c>
+      <c r="E24" s="39" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:G12"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>